<commit_message>
Docs: auditoria U07 hecha y app movil solo de consulta
</commit_message>
<xml_diff>
--- a/docs/AUDITORIA_UI_RENDIMIENTO.xlsx
+++ b/docs/AUDITORIA_UI_RENDIMIENTO.xlsx
@@ -2344,12 +2344,12 @@
       </c>
       <c r="K23" s="24" t="inlineStr">
         <is>
-          <t>Parcial</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="L23" s="23" t="inlineStr">
         <is>
-          <t>Unificados x-pagination, x-avatar, x-markdown y diálogo; pestañas aún en dos componentes.</t>
+          <t>Unificados x-pagination, x-avatar, x-markdown, diálogo y pestañas (x-tabs, variantes subrayado y píldoras) en proyecto, repositorio, PR, notificaciones e issues/PR.</t>
         </is>
       </c>
     </row>

</xml_diff>